<commit_message>
OP1188 amend spreadsheet to include Twice-monthly
</commit_message>
<xml_diff>
--- a/assets/importtemplate.xlsx
+++ b/assets/importtemplate.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
@@ -8,11 +8,11 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Instructions" sheetId="1" state="visible" r:id="rId2"/>
-    <sheet name="Contacts" sheetId="2" state="visible" r:id="rId3"/>
-    <sheet name="Venues" sheetId="3" state="visible" r:id="rId4"/>
-    <sheet name="Groups" sheetId="4" state="visible" r:id="rId5"/>
-    <sheet name="Events" sheetId="5" state="visible" r:id="rId6"/>
+    <sheet name="Instructions" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Contacts" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Venues" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Groups" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Events" sheetId="5" state="visible" r:id="rId7"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -129,7 +129,7 @@
     <t xml:space="preserve">The ‘Time’ must be one of  'Morning', 'Afternoon', 'Evening', 'All Day' or may be omitted.</t>
   </si>
   <si>
-    <t xml:space="preserve">The ‘Frequency’ must be one of  'Weekly', 'Fortnightly', 'Monthly' or may be omitted.</t>
+    <t xml:space="preserve">The ‘Frequency’ must be one of  'Weekly', 'Fortnightly', 'Monthly', 'Twice-monthly' or may be omitted.</t>
   </si>
   <si>
     <t xml:space="preserve">The ‘Venue’ must match the name of an existing Venue, or may be omitted.  New Venues must be created if necessary before importing.</t>
@@ -541,13 +541,119 @@
 </styleSheet>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office">
+  <a:themeElements>
+    <a:clrScheme name="LibreOffice">
+      <a:dk1>
+        <a:srgbClr val="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:srgbClr val="ffffff"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="000000"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="ffffff"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="18a303"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="0369a3"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="a33e03"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8e03a3"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="c99c00"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="c9211e"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000ee"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="551a8b"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme>
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:A1048576"/>
-  <sheetFormatPr defaultColWidth="12.578125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="1" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.578125" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="1" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="125.44"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="2" style="2" width="12.56"/>
@@ -822,12 +928,12 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G1"/>
-  <sheetFormatPr defaultColWidth="12.6796875" defaultRowHeight="13.2" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.6796875" defaultRowHeight="13.2" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="8" width="16"/>
   </cols>
@@ -867,12 +973,12 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:I1"/>
-  <sheetFormatPr defaultColWidth="12.6796875" defaultRowHeight="13.2" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.6796875" defaultRowHeight="13.2" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="8" width="17.21"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="8" width="16.22"/>
@@ -919,12 +1025,12 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:Q1"/>
-  <sheetFormatPr defaultColWidth="12.6796875" defaultRowHeight="13.2" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.6796875" defaultRowHeight="13.2" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="8" t="s">
@@ -991,12 +1097,12 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:K1"/>
-  <sheetFormatPr defaultColWidth="12.6796875" defaultRowHeight="13.2" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.6796875" defaultRowHeight="13.2" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="8" t="s">

</xml_diff>